<commit_message>
fix row shift and add test fort build thermal parameters
</commit_message>
<xml_diff>
--- a/src/test/resources/thermal_parameters/common_param_BP23_A_ref.xlsx
+++ b/src/test/resources/thermal_parameters/common_param_BP23_A_ref.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28521"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28528"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\ESPACES_PERSO\TZ\refonte générateur\arborescence hypothèses\thermal\technical_parameters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B1174C7-9707-4DB4-BD26-C6D53C05B99F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5093008D-0142-425B-9D59-0DC47842B74F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="261">
   <si>
     <t>Nuclear/-</t>
   </si>
@@ -607,301 +607,301 @@
     <t>30% - 37%</t>
   </si>
   <si>
+    <t>Hard coal old 2</t>
+  </si>
+  <si>
+    <t>old 2</t>
+  </si>
+  <si>
+    <t>38% - 43%</t>
+  </si>
+  <si>
+    <t>Hard coal new</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>44% - 46%</t>
+  </si>
+  <si>
+    <t>Hard coal CCS</t>
+  </si>
+  <si>
+    <t>CCS</t>
+  </si>
+  <si>
+    <t>30% - 40%</t>
+  </si>
+  <si>
+    <t>Lignite old 1</t>
+  </si>
+  <si>
+    <t>Lignite</t>
+  </si>
+  <si>
+    <t>Lignite old 2</t>
+  </si>
+  <si>
+    <t>Lignite new</t>
+  </si>
+  <si>
+    <t>Lignite CCS</t>
+  </si>
+  <si>
+    <t>Gas conventional old 1</t>
+  </si>
+  <si>
+    <t>Gas</t>
+  </si>
+  <si>
+    <t>conventional old 1</t>
+  </si>
+  <si>
+    <t>25% - 38%</t>
+  </si>
+  <si>
+    <t>Gas conventional old 2</t>
+  </si>
+  <si>
+    <t>conventional old 2</t>
+  </si>
+  <si>
+    <t>39% - 42%</t>
+  </si>
+  <si>
+    <t>CCGT old 1</t>
+  </si>
+  <si>
+    <t>33% - 44%</t>
+  </si>
+  <si>
+    <t>CCGT old 2</t>
+  </si>
+  <si>
+    <t>45% - 52%</t>
+  </si>
+  <si>
+    <t>CCGT present 1</t>
+  </si>
+  <si>
+    <t>53% - 60%</t>
+  </si>
+  <si>
+    <t>CCGT present 2</t>
+  </si>
+  <si>
+    <t>CCGT new</t>
+  </si>
+  <si>
+    <t>CCGT CCS</t>
+  </si>
+  <si>
+    <t>43% - 52%</t>
+  </si>
+  <si>
+    <t>OCGT old</t>
+  </si>
+  <si>
+    <t>35% - 38%</t>
+  </si>
+  <si>
+    <t>OCGT new</t>
+  </si>
+  <si>
+    <t>39% - 44%</t>
+  </si>
+  <si>
+    <t>Light oil</t>
+  </si>
+  <si>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>32% - 38%</t>
+  </si>
+  <si>
+    <t>Heavy oil old 1</t>
+  </si>
+  <si>
+    <t>25% - 37%</t>
+  </si>
+  <si>
+    <t>Heavy oil old 2</t>
+  </si>
+  <si>
+    <t>Oil shale old</t>
+  </si>
+  <si>
+    <t>old</t>
+  </si>
+  <si>
+    <t>28% - 33%</t>
+  </si>
+  <si>
+    <t>Oil shale new</t>
+  </si>
+  <si>
+    <t>34% - 39%</t>
+  </si>
+  <si>
+    <t>Fuel cell/Hydrogen</t>
+  </si>
+  <si>
+    <t>Fuel cell</t>
+  </si>
+  <si>
+    <t>Hydrogen</t>
+  </si>
+  <si>
+    <t>34% - 60%</t>
+  </si>
+  <si>
+    <t>Gas pcomp mid</t>
+  </si>
+  <si>
+    <t>H2</t>
+  </si>
+  <si>
+    <t>Gas pcomp peak</t>
+  </si>
+  <si>
+    <t>audit_na_cluster</t>
+  </si>
+  <si>
+    <t>Other non identified</t>
+  </si>
+  <si>
+    <t>40% - 60%</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Hard coal/old 1</t>
+  </si>
+  <si>
+    <t>Other Hard coal old 1</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Hard coal/old 2</t>
+  </si>
+  <si>
+    <t>Other Hard coal old 2</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Hard coal/new</t>
+  </si>
+  <si>
+    <t>Other Hard coal new</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Hard coal/CCS</t>
+  </si>
+  <si>
+    <t>Other Hard coal CCS</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Lignite/old 1</t>
+  </si>
+  <si>
+    <t>Other Lignite old 1</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Lignite/old 2</t>
+  </si>
+  <si>
+    <t>Other Lignite old 2</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Lignite/new</t>
+  </si>
+  <si>
+    <t>Other Lignite new</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Lignite/CCS</t>
+  </si>
+  <si>
+    <t>Other Lignite CCS</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/conventional old 1</t>
+  </si>
+  <si>
+    <t>Other Gas conventional old 1</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/conventional old 2</t>
+  </si>
+  <si>
+    <t>Other Gas conventional old 2</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/CCGT old 1</t>
+  </si>
+  <si>
+    <t>Other CCGT old 1</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/CCGT old 2</t>
+  </si>
+  <si>
+    <t>Other CCGT old 2</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/CCGT present 1</t>
+  </si>
+  <si>
+    <t>Other CCGT present 1</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/CCGT present 2</t>
+  </si>
+  <si>
+    <t>Other CCGT present 2</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/CCGT new</t>
+  </si>
+  <si>
+    <t>Other CCGT new</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Gas/OCGT old</t>
+  </si>
+  <si>
+    <t>Other OCGT old</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Light oil/-</t>
+  </si>
+  <si>
+    <t>Other Light oil</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Heavy oil/old 2</t>
+  </si>
+  <si>
+    <t>Other Heavy oil old 2</t>
+  </si>
+  <si>
+    <t>OtherNon-RES/Oil shale/old</t>
+  </si>
+  <si>
+    <t>Other Oil shale old</t>
+  </si>
+  <si>
     <t>3.3</t>
   </si>
   <si>
-    <t>Hard coal old 2</t>
-  </si>
-  <si>
-    <t>old 2</t>
-  </si>
-  <si>
-    <t>38% - 43%</t>
-  </si>
-  <si>
-    <t>Hard coal new</t>
-  </si>
-  <si>
-    <t>new</t>
-  </si>
-  <si>
-    <t>44% - 46%</t>
-  </si>
-  <si>
-    <t>Hard coal CCS</t>
-  </si>
-  <si>
-    <t>CCS</t>
-  </si>
-  <si>
-    <t>30% - 40%</t>
-  </si>
-  <si>
     <t>6.6</t>
   </si>
   <si>
-    <t>Lignite old 1</t>
-  </si>
-  <si>
-    <t>Lignite</t>
-  </si>
-  <si>
-    <t>Lignite old 2</t>
-  </si>
-  <si>
-    <t>Lignite new</t>
-  </si>
-  <si>
-    <t>Lignite CCS</t>
-  </si>
-  <si>
-    <t>Gas conventional old 1</t>
-  </si>
-  <si>
-    <t>Gas</t>
-  </si>
-  <si>
-    <t>conventional old 1</t>
-  </si>
-  <si>
-    <t>25% - 38%</t>
-  </si>
-  <si>
     <t>1.1</t>
   </si>
   <si>
-    <t>Gas conventional old 2</t>
-  </si>
-  <si>
-    <t>conventional old 2</t>
-  </si>
-  <si>
-    <t>39% - 42%</t>
-  </si>
-  <si>
-    <t>CCGT old 1</t>
-  </si>
-  <si>
-    <t>33% - 44%</t>
-  </si>
-  <si>
     <t>1.6</t>
   </si>
   <si>
-    <t>CCGT old 2</t>
-  </si>
-  <si>
-    <t>45% - 52%</t>
-  </si>
-  <si>
-    <t>CCGT present 1</t>
-  </si>
-  <si>
-    <t>53% - 60%</t>
-  </si>
-  <si>
-    <t>CCGT present 2</t>
-  </si>
-  <si>
-    <t>CCGT new</t>
-  </si>
-  <si>
-    <t>CCGT CCS</t>
-  </si>
-  <si>
-    <t>43% - 52%</t>
-  </si>
-  <si>
     <t>3.2</t>
-  </si>
-  <si>
-    <t>OCGT old</t>
-  </si>
-  <si>
-    <t>35% - 38%</t>
-  </si>
-  <si>
-    <t>OCGT new</t>
-  </si>
-  <si>
-    <t>39% - 44%</t>
-  </si>
-  <si>
-    <t>Light oil</t>
-  </si>
-  <si>
-    <t>Oil</t>
-  </si>
-  <si>
-    <t>32% - 38%</t>
-  </si>
-  <si>
-    <t>Heavy oil old 1</t>
-  </si>
-  <si>
-    <t>25% - 37%</t>
-  </si>
-  <si>
-    <t>Heavy oil old 2</t>
-  </si>
-  <si>
-    <t>Oil shale old</t>
-  </si>
-  <si>
-    <t>old</t>
-  </si>
-  <si>
-    <t>28% - 33%</t>
-  </si>
-  <si>
-    <t>Oil shale new</t>
-  </si>
-  <si>
-    <t>34% - 39%</t>
-  </si>
-  <si>
-    <t>Fuel cell/Hydrogen</t>
-  </si>
-  <si>
-    <t>Fuel cell</t>
-  </si>
-  <si>
-    <t>Hydrogen</t>
-  </si>
-  <si>
-    <t>34% - 60%</t>
-  </si>
-  <si>
-    <t>Gas pcomp mid</t>
-  </si>
-  <si>
-    <t>H2</t>
-  </si>
-  <si>
-    <t>Gas pcomp peak</t>
-  </si>
-  <si>
-    <t>audit_na_cluster</t>
-  </si>
-  <si>
-    <t>Other non identified</t>
-  </si>
-  <si>
-    <t>40% - 60%</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Hard coal/old 1</t>
-  </si>
-  <si>
-    <t>Other Hard coal old 1</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Hard coal/old 2</t>
-  </si>
-  <si>
-    <t>Other Hard coal old 2</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Hard coal/new</t>
-  </si>
-  <si>
-    <t>Other Hard coal new</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Hard coal/CCS</t>
-  </si>
-  <si>
-    <t>Other Hard coal CCS</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Lignite/old 1</t>
-  </si>
-  <si>
-    <t>Other Lignite old 1</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Lignite/old 2</t>
-  </si>
-  <si>
-    <t>Other Lignite old 2</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Lignite/new</t>
-  </si>
-  <si>
-    <t>Other Lignite new</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Lignite/CCS</t>
-  </si>
-  <si>
-    <t>Other Lignite CCS</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/conventional old 1</t>
-  </si>
-  <si>
-    <t>Other Gas conventional old 1</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/conventional old 2</t>
-  </si>
-  <si>
-    <t>Other Gas conventional old 2</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/CCGT old 1</t>
-  </si>
-  <si>
-    <t>Other CCGT old 1</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/CCGT old 2</t>
-  </si>
-  <si>
-    <t>Other CCGT old 2</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/CCGT present 1</t>
-  </si>
-  <si>
-    <t>Other CCGT present 1</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/CCGT present 2</t>
-  </si>
-  <si>
-    <t>Other CCGT present 2</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/CCGT new</t>
-  </si>
-  <si>
-    <t>Other CCGT new</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Gas/OCGT old</t>
-  </si>
-  <si>
-    <t>Other OCGT old</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Light oil/-</t>
-  </si>
-  <si>
-    <t>Other Light oil</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Heavy oil/old 2</t>
-  </si>
-  <si>
-    <t>Other Heavy oil old 2</t>
-  </si>
-  <si>
-    <t>OtherNon-RES/Oil shale/old</t>
-  </si>
-  <si>
-    <t>Other Oil shale old</t>
   </si>
 </sst>
 </file>
@@ -3163,8 +3163,8 @@
       <c r="H7" s="11">
         <v>94</v>
       </c>
-      <c r="I7" s="11" t="s">
-        <v>162</v>
+      <c r="I7" s="11">
+        <v>3.3</v>
       </c>
       <c r="J7" s="11">
         <v>8</v>
@@ -3237,7 +3237,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C8" s="11">
         <v>3</v>
@@ -3246,10 +3246,10 @@
         <v>159</v>
       </c>
       <c r="E8" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G8" s="10">
         <v>0.4</v>
@@ -3257,8 +3257,8 @@
       <c r="H8" s="11">
         <v>94</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>162</v>
+      <c r="I8" s="11">
+        <v>3.3</v>
       </c>
       <c r="J8" s="11">
         <v>6</v>
@@ -3331,7 +3331,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C9" s="11">
         <v>4</v>
@@ -3340,10 +3340,10 @@
         <v>159</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G9" s="10">
         <v>0.46</v>
@@ -3351,8 +3351,8 @@
       <c r="H9" s="11">
         <v>94</v>
       </c>
-      <c r="I9" s="11" t="s">
-        <v>162</v>
+      <c r="I9" s="11">
+        <v>3.3</v>
       </c>
       <c r="J9" s="11">
         <v>5</v>
@@ -3425,7 +3425,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C10" s="11">
         <v>5</v>
@@ -3434,10 +3434,10 @@
         <v>159</v>
       </c>
       <c r="E10" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G10" s="10">
         <v>0.38</v>
@@ -3445,8 +3445,8 @@
       <c r="H10" s="11">
         <v>9.4</v>
       </c>
-      <c r="I10" s="11" t="s">
-        <v>172</v>
+      <c r="I10" s="11">
+        <v>6.6</v>
       </c>
       <c r="J10" s="11">
         <v>7</v>
@@ -3515,13 +3515,13 @@
         <v>5</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C11" s="11">
         <v>6</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>160</v>
@@ -3535,8 +3535,8 @@
       <c r="H11" s="11">
         <v>101</v>
       </c>
-      <c r="I11" s="11" t="s">
-        <v>162</v>
+      <c r="I11" s="11">
+        <v>3.3</v>
       </c>
       <c r="J11" s="11">
         <v>11</v>
@@ -3609,19 +3609,19 @@
         <v>6</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C12" s="11">
         <v>7</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E12" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F12" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G12" s="10">
         <v>0.4</v>
@@ -3629,8 +3629,8 @@
       <c r="H12" s="11">
         <v>101</v>
       </c>
-      <c r="I12" s="11" t="s">
-        <v>162</v>
+      <c r="I12" s="11">
+        <v>3.3</v>
       </c>
       <c r="J12" s="11">
         <v>9</v>
@@ -3703,19 +3703,19 @@
         <v>7</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C13" s="11">
         <v>8</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E13" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G13" s="10">
         <v>0.46</v>
@@ -3723,8 +3723,8 @@
       <c r="H13" s="11">
         <v>101</v>
       </c>
-      <c r="I13" s="11" t="s">
-        <v>162</v>
+      <c r="I13" s="11">
+        <v>3.3</v>
       </c>
       <c r="J13" s="11">
         <v>8</v>
@@ -3797,19 +3797,19 @@
         <v>8</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C14" s="11">
         <v>9</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E14" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F14" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G14" s="10">
         <v>0.38</v>
@@ -3817,8 +3817,8 @@
       <c r="H14" s="11">
         <v>10.1</v>
       </c>
-      <c r="I14" s="11" t="s">
-        <v>172</v>
+      <c r="I14" s="11">
+        <v>6.6</v>
       </c>
       <c r="J14" s="11">
         <v>10</v>
@@ -3887,19 +3887,19 @@
         <v>9</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C15" s="11">
         <v>10</v>
       </c>
       <c r="D15" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F15" s="9" t="s">
         <v>179</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>181</v>
       </c>
       <c r="G15" s="10">
         <v>0.36</v>
@@ -3907,8 +3907,8 @@
       <c r="H15" s="11">
         <v>57</v>
       </c>
-      <c r="I15" s="11" t="s">
-        <v>182</v>
+      <c r="I15" s="11">
+        <v>1.1000000000000001</v>
       </c>
       <c r="J15" s="11">
         <v>5</v>
@@ -3981,19 +3981,19 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C16" s="11">
         <v>11</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G16" s="10">
         <v>0.41</v>
@@ -4001,8 +4001,8 @@
       <c r="H16" s="11">
         <v>57</v>
       </c>
-      <c r="I16" s="11" t="s">
-        <v>182</v>
+      <c r="I16" s="11">
+        <v>1.1000000000000001</v>
       </c>
       <c r="J16" s="11">
         <v>5</v>
@@ -4071,19 +4071,19 @@
         <v>11</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C17" s="11">
         <v>12</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G17" s="10">
         <v>0.4</v>
@@ -4091,8 +4091,8 @@
       <c r="H17" s="11">
         <v>57</v>
       </c>
-      <c r="I17" s="11" t="s">
-        <v>188</v>
+      <c r="I17" s="11">
+        <v>1.6</v>
       </c>
       <c r="J17" s="11">
         <v>3</v>
@@ -4165,19 +4165,19 @@
         <v>12</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C18" s="11">
         <v>13</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G18" s="10">
         <v>0.48</v>
@@ -4185,8 +4185,8 @@
       <c r="H18" s="11">
         <v>57</v>
       </c>
-      <c r="I18" s="11" t="s">
-        <v>188</v>
+      <c r="I18" s="11">
+        <v>1.6</v>
       </c>
       <c r="J18" s="11">
         <v>3</v>
@@ -4259,19 +4259,19 @@
         <v>22</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C19" s="11">
         <v>14</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G19" s="10">
         <v>0.56000000000000005</v>
@@ -4279,8 +4279,8 @@
       <c r="H19" s="11">
         <v>57</v>
       </c>
-      <c r="I19" s="11" t="s">
-        <v>188</v>
+      <c r="I19" s="11">
+        <v>1.6</v>
       </c>
       <c r="J19" s="11">
         <v>2</v>
@@ -4353,19 +4353,19 @@
         <v>23</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C20" s="11">
         <v>15</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G20" s="10">
         <v>0.57999999999999996</v>
@@ -4373,8 +4373,8 @@
       <c r="H20" s="11">
         <v>57</v>
       </c>
-      <c r="I20" s="11" t="s">
-        <v>188</v>
+      <c r="I20" s="11">
+        <v>1.6</v>
       </c>
       <c r="J20" s="11">
         <v>2</v>
@@ -4447,19 +4447,19 @@
         <v>13</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C21" s="11">
         <v>16</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G21" s="10">
         <v>0.6</v>
@@ -4467,8 +4467,8 @@
       <c r="H21" s="11">
         <v>57</v>
       </c>
-      <c r="I21" s="11" t="s">
-        <v>188</v>
+      <c r="I21" s="11">
+        <v>1.6</v>
       </c>
       <c r="J21" s="11">
         <v>2</v>
@@ -4541,19 +4541,19 @@
         <v>14</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C22" s="11">
         <v>17</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="G22" s="10">
         <v>0.51</v>
@@ -4561,8 +4561,8 @@
       <c r="H22" s="11">
         <v>5.7</v>
       </c>
-      <c r="I22" s="11" t="s">
-        <v>197</v>
+      <c r="I22" s="11">
+        <v>3.2</v>
       </c>
       <c r="J22" s="11">
         <v>4</v>
@@ -4631,19 +4631,19 @@
         <v>15</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C23" s="11">
         <v>18</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="G23" s="10">
         <v>0.35</v>
@@ -4651,8 +4651,8 @@
       <c r="H23" s="11">
         <v>57</v>
       </c>
-      <c r="I23" s="11" t="s">
-        <v>188</v>
+      <c r="I23" s="11">
+        <v>1.6</v>
       </c>
       <c r="J23" s="11">
         <v>1</v>
@@ -4725,19 +4725,19 @@
         <v>16</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C24" s="11">
         <v>19</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G24" s="10">
         <v>0.42</v>
@@ -4745,8 +4745,8 @@
       <c r="H24" s="11">
         <v>57</v>
       </c>
-      <c r="I24" s="11" t="s">
-        <v>188</v>
+      <c r="I24" s="11">
+        <v>1.6</v>
       </c>
       <c r="J24" s="11">
         <v>1</v>
@@ -4819,19 +4819,19 @@
         <v>17</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C25" s="11">
         <v>20</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>156</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G25" s="10">
         <v>0.35</v>
@@ -4839,8 +4839,8 @@
       <c r="H25" s="11">
         <v>78</v>
       </c>
-      <c r="I25" s="11" t="s">
-        <v>182</v>
+      <c r="I25" s="11">
+        <v>1.1000000000000001</v>
       </c>
       <c r="J25" s="11">
         <v>1</v>
@@ -4913,19 +4913,19 @@
         <v>18</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C26" s="11">
         <v>21</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>160</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="G26" s="10">
         <v>0.35</v>
@@ -4933,8 +4933,8 @@
       <c r="H26" s="11">
         <v>78</v>
       </c>
-      <c r="I26" s="11" t="s">
-        <v>162</v>
+      <c r="I26" s="11">
+        <v>3.3</v>
       </c>
       <c r="J26" s="11">
         <v>3</v>
@@ -5007,19 +5007,19 @@
         <v>19</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C27" s="11">
         <v>22</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E27" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F27" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G27" s="10">
         <v>0.4</v>
@@ -5027,8 +5027,8 @@
       <c r="H27" s="11">
         <v>78</v>
       </c>
-      <c r="I27" s="11" t="s">
-        <v>162</v>
+      <c r="I27" s="11">
+        <v>3.3</v>
       </c>
       <c r="J27" s="11">
         <v>3</v>
@@ -5101,19 +5101,19 @@
         <v>20</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C28" s="11">
         <v>23</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="G28" s="10">
         <v>0.28999999999999998</v>
@@ -5121,8 +5121,8 @@
       <c r="H28" s="11">
         <v>100</v>
       </c>
-      <c r="I28" s="11" t="s">
-        <v>162</v>
+      <c r="I28" s="11">
+        <v>3.3</v>
       </c>
       <c r="J28" s="11">
         <v>11</v>
@@ -5191,19 +5191,19 @@
         <v>21</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C29" s="11">
         <v>24</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="G29" s="10">
         <v>0.39</v>
@@ -5211,8 +5211,8 @@
       <c r="H29" s="11">
         <v>100</v>
       </c>
-      <c r="I29" s="11" t="s">
-        <v>162</v>
+      <c r="I29" s="11">
+        <v>3.3</v>
       </c>
       <c r="J29" s="11">
         <v>8</v>
@@ -5278,22 +5278,22 @@
     </row>
     <row r="30" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A30" s="8" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C30" s="11">
         <v>25</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="G30" s="10">
         <v>0.6</v>
@@ -5375,19 +5375,19 @@
         <v>13</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C31" s="11">
         <v>26</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G31" s="10">
         <v>0.6</v>
@@ -5395,8 +5395,8 @@
       <c r="H31" s="11">
         <v>57</v>
       </c>
-      <c r="I31" s="11" t="s">
-        <v>188</v>
+      <c r="I31" s="11">
+        <v>1.6</v>
       </c>
       <c r="J31" s="11">
         <v>2</v>
@@ -5469,19 +5469,19 @@
         <v>16</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C32" s="11">
         <v>27</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G32" s="10">
         <v>0.42</v>
@@ -5489,8 +5489,8 @@
       <c r="H32" s="11">
         <v>57</v>
       </c>
-      <c r="I32" s="11" t="s">
-        <v>188</v>
+      <c r="I32" s="11">
+        <v>1.6</v>
       </c>
       <c r="J32" s="11">
         <v>1</v>
@@ -5560,22 +5560,22 @@
     </row>
     <row r="33" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A33" s="8" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C33" s="11">
         <v>16</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="G33" s="10">
         <v>0.5</v>
@@ -5583,8 +5583,8 @@
       <c r="H33" s="11">
         <v>57</v>
       </c>
-      <c r="I33" s="11" t="s">
-        <v>188</v>
+      <c r="I33" s="11">
+        <v>1.6</v>
       </c>
       <c r="J33" s="11">
         <v>2</v>
@@ -5654,10 +5654,10 @@
     </row>
     <row r="34" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A34" s="8" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C34" s="11">
         <v>2</v>
@@ -5677,8 +5677,8 @@
       <c r="H34" s="11">
         <v>94</v>
       </c>
-      <c r="I34" s="11" t="s">
-        <v>162</v>
+      <c r="I34" s="11">
+        <v>3.3</v>
       </c>
       <c r="J34" s="11">
         <v>8</v>
@@ -5748,10 +5748,10 @@
     </row>
     <row r="35" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A35" s="8" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C35" s="11">
         <v>3</v>
@@ -5760,10 +5760,10 @@
         <v>159</v>
       </c>
       <c r="E35" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G35" s="10">
         <v>0.4</v>
@@ -5771,8 +5771,8 @@
       <c r="H35" s="11">
         <v>94</v>
       </c>
-      <c r="I35" s="11" t="s">
-        <v>162</v>
+      <c r="I35" s="11">
+        <v>3.3</v>
       </c>
       <c r="J35" s="11">
         <v>6</v>
@@ -5842,10 +5842,10 @@
     </row>
     <row r="36" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A36" s="8" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="C36" s="11">
         <v>4</v>
@@ -5854,10 +5854,10 @@
         <v>159</v>
       </c>
       <c r="E36" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F36" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G36" s="10">
         <v>0.46</v>
@@ -5865,8 +5865,8 @@
       <c r="H36" s="11">
         <v>94</v>
       </c>
-      <c r="I36" s="11" t="s">
-        <v>162</v>
+      <c r="I36" s="11">
+        <v>3.3</v>
       </c>
       <c r="J36" s="11">
         <v>5</v>
@@ -5936,10 +5936,10 @@
     </row>
     <row r="37" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A37" s="8" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="C37" s="11">
         <v>5</v>
@@ -5948,10 +5948,10 @@
         <v>159</v>
       </c>
       <c r="E37" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F37" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G37" s="10">
         <v>0.38</v>
@@ -5959,8 +5959,8 @@
       <c r="H37" s="11">
         <v>9.4</v>
       </c>
-      <c r="I37" s="11" t="s">
-        <v>172</v>
+      <c r="I37" s="11">
+        <v>6.6</v>
       </c>
       <c r="J37" s="11">
         <v>7</v>
@@ -6026,16 +6026,16 @@
     </row>
     <row r="38" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A38" s="8" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="C38" s="11">
         <v>6</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E38" s="8" t="s">
         <v>160</v>
@@ -6049,8 +6049,8 @@
       <c r="H38" s="11">
         <v>101</v>
       </c>
-      <c r="I38" s="11" t="s">
-        <v>162</v>
+      <c r="I38" s="11">
+        <v>3.3</v>
       </c>
       <c r="J38" s="11">
         <v>11</v>
@@ -6120,22 +6120,22 @@
     </row>
     <row r="39" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A39" s="8" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C39" s="11">
         <v>7</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E39" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F39" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G39" s="10">
         <v>0.4</v>
@@ -6143,8 +6143,8 @@
       <c r="H39" s="11">
         <v>101</v>
       </c>
-      <c r="I39" s="11" t="s">
-        <v>162</v>
+      <c r="I39" s="11">
+        <v>3.3</v>
       </c>
       <c r="J39" s="11">
         <v>9</v>
@@ -6214,22 +6214,22 @@
     </row>
     <row r="40" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A40" s="8" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C40" s="11">
         <v>8</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E40" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F40" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G40" s="10">
         <v>0.46</v>
@@ -6237,8 +6237,8 @@
       <c r="H40" s="11">
         <v>101</v>
       </c>
-      <c r="I40" s="11" t="s">
-        <v>162</v>
+      <c r="I40" s="11">
+        <v>3.3</v>
       </c>
       <c r="J40" s="11">
         <v>8</v>
@@ -6308,22 +6308,22 @@
     </row>
     <row r="41" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A41" s="8" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C41" s="11">
         <v>9</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E41" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F41" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G41" s="10">
         <v>0.38</v>
@@ -6331,8 +6331,8 @@
       <c r="H41" s="11">
         <v>10.1</v>
       </c>
-      <c r="I41" s="11" t="s">
-        <v>172</v>
+      <c r="I41" s="11">
+        <v>6.6</v>
       </c>
       <c r="J41" s="11">
         <v>10</v>
@@ -6398,22 +6398,22 @@
     </row>
     <row r="42" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A42" s="8" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C42" s="11">
         <v>10</v>
       </c>
       <c r="D42" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F42" s="9" t="s">
         <v>179</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>181</v>
       </c>
       <c r="G42" s="10">
         <v>0.36</v>
@@ -6421,8 +6421,8 @@
       <c r="H42" s="11">
         <v>57</v>
       </c>
-      <c r="I42" s="11" t="s">
-        <v>182</v>
+      <c r="I42" s="11">
+        <v>1.1000000000000001</v>
       </c>
       <c r="J42" s="11">
         <v>5</v>
@@ -6492,22 +6492,22 @@
     </row>
     <row r="43" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A43" s="8" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C43" s="11">
         <v>11</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G43" s="10">
         <v>0.41</v>
@@ -6515,8 +6515,8 @@
       <c r="H43" s="11">
         <v>57</v>
       </c>
-      <c r="I43" s="11" t="s">
-        <v>182</v>
+      <c r="I43" s="11">
+        <v>1.1000000000000001</v>
       </c>
       <c r="J43" s="11">
         <v>5</v>
@@ -6582,22 +6582,22 @@
     </row>
     <row r="44" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A44" s="8" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C44" s="11">
         <v>12</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G44" s="10">
         <v>0.4</v>
@@ -6605,8 +6605,8 @@
       <c r="H44" s="11">
         <v>57</v>
       </c>
-      <c r="I44" s="11" t="s">
-        <v>188</v>
+      <c r="I44" s="11">
+        <v>1.6</v>
       </c>
       <c r="J44" s="11">
         <v>3</v>
@@ -6676,22 +6676,22 @@
     </row>
     <row r="45" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A45" s="8" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="C45" s="11">
         <v>13</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G45" s="10">
         <v>0.48</v>
@@ -6699,8 +6699,8 @@
       <c r="H45" s="11">
         <v>57</v>
       </c>
-      <c r="I45" s="11" t="s">
-        <v>188</v>
+      <c r="I45" s="11">
+        <v>1.6</v>
       </c>
       <c r="J45" s="11">
         <v>3</v>
@@ -6770,22 +6770,22 @@
     </row>
     <row r="46" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A46" s="8" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C46" s="11">
         <v>14</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G46" s="10">
         <v>0.56000000000000005</v>
@@ -6793,8 +6793,8 @@
       <c r="H46" s="11">
         <v>57</v>
       </c>
-      <c r="I46" s="11" t="s">
-        <v>188</v>
+      <c r="I46" s="11">
+        <v>1.6</v>
       </c>
       <c r="J46" s="11">
         <v>2</v>
@@ -6864,22 +6864,22 @@
     </row>
     <row r="47" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A47" s="8" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C47" s="11">
         <v>15</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G47" s="10">
         <v>0.57999999999999996</v>
@@ -6887,8 +6887,8 @@
       <c r="H47" s="11">
         <v>57</v>
       </c>
-      <c r="I47" s="11" t="s">
-        <v>188</v>
+      <c r="I47" s="11">
+        <v>1.6</v>
       </c>
       <c r="J47" s="11">
         <v>2</v>
@@ -6958,22 +6958,22 @@
     </row>
     <row r="48" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A48" s="8" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C48" s="11">
         <v>16</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G48" s="10">
         <v>0.6</v>
@@ -6981,8 +6981,8 @@
       <c r="H48" s="11">
         <v>57</v>
       </c>
-      <c r="I48" s="11" t="s">
-        <v>188</v>
+      <c r="I48" s="11">
+        <v>1.6</v>
       </c>
       <c r="J48" s="11">
         <v>2</v>
@@ -7052,22 +7052,22 @@
     </row>
     <row r="49" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A49" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C49" s="11">
         <v>18</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="G49" s="10">
         <v>0.35</v>
@@ -7075,8 +7075,8 @@
       <c r="H49" s="11">
         <v>57</v>
       </c>
-      <c r="I49" s="11" t="s">
-        <v>188</v>
+      <c r="I49" s="11">
+        <v>1.6</v>
       </c>
       <c r="J49" s="11">
         <v>1</v>
@@ -7146,22 +7146,22 @@
     </row>
     <row r="50" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A50" s="8" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C50" s="11">
         <v>20</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>156</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G50" s="10">
         <v>0.35</v>
@@ -7169,8 +7169,8 @@
       <c r="H50" s="11">
         <v>78</v>
       </c>
-      <c r="I50" s="11" t="s">
-        <v>182</v>
+      <c r="I50" s="11">
+        <v>1.1000000000000001</v>
       </c>
       <c r="J50" s="11">
         <v>1</v>
@@ -7240,22 +7240,22 @@
     </row>
     <row r="51" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A51" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C51" s="11">
         <v>22</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E51" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F51" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G51" s="10">
         <v>0.4</v>
@@ -7263,8 +7263,8 @@
       <c r="H51" s="11">
         <v>78</v>
       </c>
-      <c r="I51" s="11" t="s">
-        <v>162</v>
+      <c r="I51" s="11">
+        <v>3.3</v>
       </c>
       <c r="J51" s="11">
         <v>3</v>
@@ -7334,22 +7334,22 @@
     </row>
     <row r="52" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A52" s="8" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="C52" s="11">
         <v>23</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="G52" s="10">
         <v>0.28999999999999998</v>
@@ -7357,8 +7357,8 @@
       <c r="H52" s="11">
         <v>100</v>
       </c>
-      <c r="I52" s="11" t="s">
-        <v>162</v>
+      <c r="I52" s="11">
+        <v>3.3</v>
       </c>
       <c r="J52" s="11">
         <v>11</v>
@@ -7934,7 +7934,7 @@
         <v>94</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J7" s="11">
         <v>8</v>
@@ -8007,7 +8007,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C8" s="11">
         <v>3</v>
@@ -8016,10 +8016,10 @@
         <v>159</v>
       </c>
       <c r="E8" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G8" s="10">
         <v>0.4</v>
@@ -8028,7 +8028,7 @@
         <v>94</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J8" s="11">
         <v>6</v>
@@ -8101,7 +8101,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C9" s="11">
         <v>4</v>
@@ -8110,10 +8110,10 @@
         <v>159</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G9" s="10">
         <v>0.46</v>
@@ -8122,7 +8122,7 @@
         <v>94</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J9" s="11">
         <v>5</v>
@@ -8195,7 +8195,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C10" s="11">
         <v>5</v>
@@ -8204,10 +8204,10 @@
         <v>159</v>
       </c>
       <c r="E10" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G10" s="10">
         <v>0.38</v>
@@ -8216,7 +8216,7 @@
         <v>9.4</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>172</v>
+        <v>257</v>
       </c>
       <c r="J10" s="11">
         <v>7</v>
@@ -8285,13 +8285,13 @@
         <v>5</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C11" s="11">
         <v>6</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>160</v>
@@ -8306,7 +8306,7 @@
         <v>101</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J11" s="11">
         <v>11</v>
@@ -8379,19 +8379,19 @@
         <v>6</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C12" s="11">
         <v>7</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E12" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F12" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G12" s="10">
         <v>0.4</v>
@@ -8400,7 +8400,7 @@
         <v>101</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J12" s="11">
         <v>9</v>
@@ -8473,19 +8473,19 @@
         <v>7</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C13" s="11">
         <v>8</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E13" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G13" s="10">
         <v>0.46</v>
@@ -8494,7 +8494,7 @@
         <v>101</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J13" s="11">
         <v>8</v>
@@ -8567,19 +8567,19 @@
         <v>8</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C14" s="11">
         <v>9</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E14" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F14" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G14" s="10">
         <v>0.38</v>
@@ -8588,7 +8588,7 @@
         <v>10.1</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>172</v>
+        <v>257</v>
       </c>
       <c r="J14" s="11">
         <v>10</v>
@@ -8657,19 +8657,19 @@
         <v>9</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C15" s="11">
         <v>10</v>
       </c>
       <c r="D15" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F15" s="9" t="s">
         <v>179</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>181</v>
       </c>
       <c r="G15" s="10">
         <v>0.36</v>
@@ -8678,7 +8678,7 @@
         <v>57</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>182</v>
+        <v>258</v>
       </c>
       <c r="J15" s="11">
         <v>5</v>
@@ -8751,19 +8751,19 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C16" s="11">
         <v>11</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G16" s="10">
         <v>0.41</v>
@@ -8772,7 +8772,7 @@
         <v>57</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>182</v>
+        <v>258</v>
       </c>
       <c r="J16" s="11">
         <v>5</v>
@@ -8841,19 +8841,19 @@
         <v>11</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C17" s="11">
         <v>12</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G17" s="10">
         <v>0.4</v>
@@ -8862,7 +8862,7 @@
         <v>57</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J17" s="11">
         <v>3</v>
@@ -8935,19 +8935,19 @@
         <v>12</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C18" s="11">
         <v>13</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G18" s="10">
         <v>0.48</v>
@@ -8956,7 +8956,7 @@
         <v>57</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J18" s="11">
         <v>3</v>
@@ -9029,19 +9029,19 @@
         <v>22</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C19" s="11">
         <v>14</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G19" s="10">
         <v>0.56000000000000005</v>
@@ -9050,7 +9050,7 @@
         <v>57</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J19" s="11">
         <v>2</v>
@@ -9123,19 +9123,19 @@
         <v>23</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C20" s="11">
         <v>15</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G20" s="10">
         <v>0.57999999999999996</v>
@@ -9144,7 +9144,7 @@
         <v>57</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J20" s="11">
         <v>2</v>
@@ -9217,19 +9217,19 @@
         <v>13</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C21" s="11">
         <v>16</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G21" s="10">
         <v>0.6</v>
@@ -9238,7 +9238,7 @@
         <v>57</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J21" s="11">
         <v>2</v>
@@ -9311,19 +9311,19 @@
         <v>14</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C22" s="11">
         <v>17</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="G22" s="10">
         <v>0.51</v>
@@ -9332,7 +9332,7 @@
         <v>5.7</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>197</v>
+        <v>260</v>
       </c>
       <c r="J22" s="11">
         <v>4</v>
@@ -9401,19 +9401,19 @@
         <v>15</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C23" s="11">
         <v>18</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="G23" s="10">
         <v>0.35</v>
@@ -9422,7 +9422,7 @@
         <v>57</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J23" s="11">
         <v>1</v>
@@ -9495,19 +9495,19 @@
         <v>16</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C24" s="11">
         <v>19</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G24" s="10">
         <v>0.42</v>
@@ -9516,7 +9516,7 @@
         <v>57</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J24" s="11">
         <v>1</v>
@@ -9589,19 +9589,19 @@
         <v>17</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C25" s="11">
         <v>20</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>156</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G25" s="10">
         <v>0.35</v>
@@ -9610,7 +9610,7 @@
         <v>78</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>182</v>
+        <v>258</v>
       </c>
       <c r="J25" s="11">
         <v>1</v>
@@ -9683,19 +9683,19 @@
         <v>18</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C26" s="11">
         <v>21</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>160</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="G26" s="10">
         <v>0.35</v>
@@ -9704,7 +9704,7 @@
         <v>78</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J26" s="11">
         <v>3</v>
@@ -9777,19 +9777,19 @@
         <v>19</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C27" s="11">
         <v>22</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E27" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F27" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G27" s="10">
         <v>0.4</v>
@@ -9798,7 +9798,7 @@
         <v>78</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J27" s="11">
         <v>3</v>
@@ -9871,19 +9871,19 @@
         <v>20</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C28" s="11">
         <v>23</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="G28" s="10">
         <v>0.28999999999999998</v>
@@ -9892,7 +9892,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J28" s="11">
         <v>11</v>
@@ -9961,19 +9961,19 @@
         <v>21</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C29" s="11">
         <v>24</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="G29" s="10">
         <v>0.39</v>
@@ -9982,7 +9982,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J29" s="11">
         <v>8</v>
@@ -10048,22 +10048,22 @@
     </row>
     <row r="30" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A30" s="8" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C30" s="11">
         <v>25</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="G30" s="10">
         <v>0.6</v>
@@ -10145,19 +10145,19 @@
         <v>13</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C31" s="11">
         <v>26</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G31" s="10">
         <v>0.6</v>
@@ -10166,7 +10166,7 @@
         <v>57</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J31" s="11">
         <v>2</v>
@@ -10239,19 +10239,19 @@
         <v>16</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C32" s="11">
         <v>27</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G32" s="10">
         <v>0.42</v>
@@ -10260,7 +10260,7 @@
         <v>57</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J32" s="11">
         <v>1</v>
@@ -10330,22 +10330,22 @@
     </row>
     <row r="33" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A33" s="8" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C33" s="11">
         <v>16</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="G33" s="10">
         <v>0.5</v>
@@ -10354,7 +10354,7 @@
         <v>57</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J33" s="11">
         <v>2</v>
@@ -10424,10 +10424,10 @@
     </row>
     <row r="34" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A34" s="8" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C34" s="11">
         <v>2</v>
@@ -10448,7 +10448,7 @@
         <v>94</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J34" s="11">
         <v>8</v>
@@ -10518,10 +10518,10 @@
     </row>
     <row r="35" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A35" s="8" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C35" s="11">
         <v>3</v>
@@ -10530,10 +10530,10 @@
         <v>159</v>
       </c>
       <c r="E35" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G35" s="10">
         <v>0.4</v>
@@ -10542,7 +10542,7 @@
         <v>94</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J35" s="11">
         <v>6</v>
@@ -10612,10 +10612,10 @@
     </row>
     <row r="36" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A36" s="8" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="C36" s="11">
         <v>4</v>
@@ -10624,10 +10624,10 @@
         <v>159</v>
       </c>
       <c r="E36" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F36" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G36" s="10">
         <v>0.46</v>
@@ -10636,7 +10636,7 @@
         <v>94</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J36" s="11">
         <v>5</v>
@@ -10706,10 +10706,10 @@
     </row>
     <row r="37" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A37" s="8" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="C37" s="11">
         <v>5</v>
@@ -10718,10 +10718,10 @@
         <v>159</v>
       </c>
       <c r="E37" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F37" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G37" s="10">
         <v>0.38</v>
@@ -10730,7 +10730,7 @@
         <v>9.4</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>172</v>
+        <v>257</v>
       </c>
       <c r="J37" s="11">
         <v>7</v>
@@ -10796,16 +10796,16 @@
     </row>
     <row r="38" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A38" s="8" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="C38" s="11">
         <v>6</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E38" s="8" t="s">
         <v>160</v>
@@ -10820,7 +10820,7 @@
         <v>101</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J38" s="11">
         <v>11</v>
@@ -10890,22 +10890,22 @@
     </row>
     <row r="39" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A39" s="8" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C39" s="11">
         <v>7</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E39" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F39" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G39" s="10">
         <v>0.4</v>
@@ -10914,7 +10914,7 @@
         <v>101</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J39" s="11">
         <v>9</v>
@@ -10984,22 +10984,22 @@
     </row>
     <row r="40" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A40" s="8" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C40" s="11">
         <v>8</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E40" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F40" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="G40" s="10">
         <v>0.46</v>
@@ -11008,7 +11008,7 @@
         <v>101</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J40" s="11">
         <v>8</v>
@@ -11078,22 +11078,22 @@
     </row>
     <row r="41" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A41" s="8" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C41" s="11">
         <v>9</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E41" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F41" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="G41" s="10">
         <v>0.38</v>
@@ -11102,7 +11102,7 @@
         <v>10.1</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>172</v>
+        <v>257</v>
       </c>
       <c r="J41" s="11">
         <v>10</v>
@@ -11168,22 +11168,22 @@
     </row>
     <row r="42" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A42" s="8" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C42" s="11">
         <v>10</v>
       </c>
       <c r="D42" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F42" s="9" t="s">
         <v>179</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>181</v>
       </c>
       <c r="G42" s="10">
         <v>0.36</v>
@@ -11192,7 +11192,7 @@
         <v>57</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>182</v>
+        <v>258</v>
       </c>
       <c r="J42" s="11">
         <v>5</v>
@@ -11262,22 +11262,22 @@
     </row>
     <row r="43" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A43" s="8" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C43" s="11">
         <v>11</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G43" s="10">
         <v>0.41</v>
@@ -11286,7 +11286,7 @@
         <v>57</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>182</v>
+        <v>258</v>
       </c>
       <c r="J43" s="11">
         <v>5</v>
@@ -11352,22 +11352,22 @@
     </row>
     <row r="44" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A44" s="8" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C44" s="11">
         <v>12</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G44" s="10">
         <v>0.4</v>
@@ -11376,7 +11376,7 @@
         <v>57</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J44" s="11">
         <v>3</v>
@@ -11446,22 +11446,22 @@
     </row>
     <row r="45" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A45" s="8" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="C45" s="11">
         <v>13</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G45" s="10">
         <v>0.48</v>
@@ -11470,7 +11470,7 @@
         <v>57</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J45" s="11">
         <v>3</v>
@@ -11540,22 +11540,22 @@
     </row>
     <row r="46" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A46" s="8" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C46" s="11">
         <v>14</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G46" s="10">
         <v>0.56000000000000005</v>
@@ -11564,7 +11564,7 @@
         <v>57</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J46" s="11">
         <v>2</v>
@@ -11634,22 +11634,22 @@
     </row>
     <row r="47" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A47" s="8" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C47" s="11">
         <v>15</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G47" s="10">
         <v>0.57999999999999996</v>
@@ -11658,7 +11658,7 @@
         <v>57</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J47" s="11">
         <v>2</v>
@@ -11728,22 +11728,22 @@
     </row>
     <row r="48" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A48" s="8" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C48" s="11">
         <v>16</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="G48" s="10">
         <v>0.6</v>
@@ -11752,7 +11752,7 @@
         <v>57</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J48" s="11">
         <v>2</v>
@@ -11822,22 +11822,22 @@
     </row>
     <row r="49" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A49" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C49" s="11">
         <v>18</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="G49" s="10">
         <v>0.35</v>
@@ -11846,7 +11846,7 @@
         <v>57</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
       <c r="J49" s="11">
         <v>1</v>
@@ -11916,22 +11916,22 @@
     </row>
     <row r="50" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A50" s="8" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C50" s="11">
         <v>20</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>156</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G50" s="10">
         <v>0.35</v>
@@ -11940,7 +11940,7 @@
         <v>78</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>182</v>
+        <v>258</v>
       </c>
       <c r="J50" s="11">
         <v>1</v>
@@ -12010,22 +12010,22 @@
     </row>
     <row r="51" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A51" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C51" s="11">
         <v>22</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E51" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F51" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="G51" s="10">
         <v>0.4</v>
@@ -12034,7 +12034,7 @@
         <v>78</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J51" s="11">
         <v>3</v>
@@ -12104,22 +12104,22 @@
     </row>
     <row r="52" spans="1:34" ht="15" customHeight="1" thickBot="1">
       <c r="A52" s="8" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="C52" s="11">
         <v>23</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="G52" s="10">
         <v>0.28999999999999998</v>
@@ -12128,7 +12128,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="J52" s="11">
         <v>11</v>

</xml_diff>